<commit_message>
Unify sync products flow
</commit_message>
<xml_diff>
--- a/stock-sync/tests/fixtures/sample-vininova.xlsx
+++ b/stock-sync/tests/fixtures/sample-vininova.xlsx
@@ -1,19 +1,11 @@
-
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
-</file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
-    <t>NR_REF</t>
+    <t>NR REF</t>
   </si>
   <si>
-    <t>KOD_KRESKOWY</t>
+    <t>KOD KRESKOWY</t>
   </si>
   <si>
     <t>STR. W KAT.</t>

</xml_diff>